<commit_message>
Add WordMaster 2000 batch 1 (words 51-300) and the builder
- Words 51-300: VRB-051..VRB-250 and PHR-001..PHR-050 in the 56-column
  format, with a Corrections sheet listing 15 replaced mistake examples
- Sample (1-50) rebuilt: empty synonym/antonym cells now say so
- tools/: build script plus the hand-written fields, so later batches
  can be built in any session

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NoC3WZ9app4HCpgkAbzcVk
</commit_message>
<xml_diff>
--- a/content/wordmaster-2000/WordMaster2000_Sample_Words_1-50.xlsx
+++ b/content/wordmaster-2000/WordMaster2000_Sample_Words_1-50.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Words 1–50 (sample)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Words 1–50" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Corrections" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Words 1–50 (sample)'!$A$2:$BD$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Words 1–50'!$A$2:$BD$52</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -125,7 +126,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -198,6 +199,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -583,7 +585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -592,76 +594,76 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>WordMaster 2000 — Sample: words 1–50</t>
+          <t>WordMaster 2000 — Batch: words 1–50</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>What this is: the first 50 of the planned 2,000 non-noun words, in the 56-column format (the 54-column WordMaster reference + 2 new columns). This is a sample to check quality and format before the other 1,950 are built.</t>
+          <t>What this is: words 1–50 of the planned 2,000 non-noun words, in the 56-column format (the 54-column WordMaster reference + 2 new columns). Same format as the 50-word sample.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Contents: 50 words from the Speak Sarthi app, in the app's own order.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>The 2 new columns (orange headers, marked ★NEW):</t>
-        </is>
-      </c>
+      <c r="A4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>• Action Sequence (Before → During → After) — in section 2. Every word in this sample is a verb. For non-verbs this column will be left blank.</t>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>The 2 new columns (orange headers, marked ★NEW):</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>• Spelling Tip — in section 3, next to Pronunciation Tip.</t>
+          <t>• Action Sequence (Before → During → After) — in section 2. Filled for verbs and phrasal verbs; it will be blank for adjectives, adverbs and other non-verbs.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Both come from the Premium Flashcard Master Specification.</t>
+          <t>• Spelling Tip — in section 3, next to Pronunciation Tip.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Both come from the Premium Flashcard Master Specification.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Where each field came from:</t>
-        </is>
-      </c>
+      <c r="A9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>• Taken from the Speak Sarthi app content (words 1–1000): IPA, syllable break, Hindi pronunciation and meaning, category, register, explanations, examples, collocations, phrasal verbs, grammar pattern, common mistake, etymology, root, word family, mnemonic, visual association, emotion, synonyms, antonyms, related words, tone, mini conversation, real-life lines, and all quiz items (MCQ, fill-in, find &amp; fix, translate). Spelling tip is also from there.</t>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Where each field came from:</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>• Newly written for this file: Word Forms, Why It's Wrong, Memory Trick, Usage Tip, Write Your Own Sentence (now specific to each word), Action Sequence, Confusing Word and Difference Explained.</t>
+          <t>• Taken from the Speak Sarthi app content: IPA, syllable break, Hindi pronunciation and meaning, category, register, explanations, examples, collocations, phrasal verbs, grammar pattern, common mistake, etymology, root, word family, mnemonic, visual association, emotion, synonyms, antonyms, related words, tone, mini conversation, real-life lines, spelling tip, and all quiz items.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>• Confusing Word / Difference Explained were rewritten, not copied: several app entries compared a word with its own past tense (understand ≠ understood) or with an unrelated sound-alike.</t>
+          <t>• Newly written for this file: Word Forms, Why It's Wrong, Memory Trick, Usage Tip, Write Your Own Sentence, Action Sequence, Confusing Word and Difference Explained.</t>
         </is>
       </c>
     </row>
@@ -675,31 +677,38 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>• AI-estimated, not from a corpus: CEFR level, frequency, importance.</t>
+          <t>• Common Mistake / Correct Version were replaced for the words listed on the 'Corrections' sheet, where the app's example was not a real error or the correction changed the meaning.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>• Real-life lines are illustrative. They are not real quotes from any film, news outlet or person.</t>
+          <t>• AI-estimated, not from a corpus: CEFR level, frequency, importance.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>• Real-life lines are illustrative. They are not real quotes from any film, news outlet or person.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Word IDs: kept from the Speak Sarthi app (VRB-001 …) so rows can be matched back to the app.</t>
-        </is>
-      </c>
+      <c r="A17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Spaced repetition plan: Day 1 → 3 → 7 → 14 → 30, same as the 910-word workbook. (The Premium spec says Day 15; say if you want that instead.)</t>
+          <t>Word IDs: kept from the Speak Sarthi app (VRB-…, PHR-…) so rows can be matched back to the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Spaced repetition plan: Day 1 → 3 → 7 → 14 → 30, same as the 910-word workbook.</t>
         </is>
       </c>
     </row>
@@ -15112,4 +15121,58 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="30" t="inlineStr">
+        <is>
+          <t>Word ID</t>
+        </is>
+      </c>
+      <c r="B1" s="30" t="inlineStr">
+        <is>
+          <t>Word</t>
+        </is>
+      </c>
+      <c r="C1" s="30" t="inlineStr">
+        <is>
+          <t>App's original mistake</t>
+        </is>
+      </c>
+      <c r="D1" s="30" t="inlineStr">
+        <is>
+          <t>App's original correction</t>
+        </is>
+      </c>
+      <c r="E1" s="30" t="inlineStr">
+        <is>
+          <t>New mistake</t>
+        </is>
+      </c>
+      <c r="F1" s="30" t="inlineStr">
+        <is>
+          <t>New correction</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>